<commit_message>
Looked at new data
</commit_message>
<xml_diff>
--- a/data/Session 10/Power variation/Powers.xlsx
+++ b/data/Session 10/Power variation/Powers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ilyag\Desktop\G\Offline\Code\Y3LaserSpec\data\Session 10\Power variation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F082E4F-0565-4D8C-A88B-28F5C7732B75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26FFD1C2-252C-4C51-BE8D-E928B638007B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6828" yWindow="1500" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -385,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -463,6 +463,46 @@
         <v>648.4</v>
       </c>
     </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>549.79999999999995</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>451.4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>349.3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>248.6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>153.4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>68.2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>117.6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>28.71</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>